<commit_message>
vault backup: 2026-10-26 23:50:59
</commit_message>
<xml_diff>
--- a/02_Areas/工作经历/鑫犇电子有限公司/04_行政部/人事/能力与培训模板.xlsx
+++ b/02_Areas/工作经历/鑫犇电子有限公司/04_行政部/人事/能力与培训模板.xlsx
@@ -1,18 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="岗位能力矩阵" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="培训记录" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="培训模块与部门确认" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="岗位能力矩阵" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="培训记录" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'岗位能力矩阵'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'培训记录'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'培训模块与部门确认'!$A$1:$L$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'培训模块与部门确认'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'岗位能力矩阵'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'培训记录'!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -21,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +40,23 @@
       <i val="1"/>
       <color rgb="007F6000"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +71,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -83,6 +111,27 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -162,7 +211,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_岗位能力矩阵" displayName="T_岗位能力矩阵" ref="A1:K2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_培训模块与部门确认" displayName="T_培训模块与部门确认" ref="A1:L12" headerRowCount="1">
+  <autoFilter ref="A1:L12"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="模块编号"/>
+    <tableColumn id="2" name="培训模块"/>
+    <tableColumn id="3" name="适用对象（初稿）"/>
+    <tableColumn id="4" name="通用目标/内容（部门需修订）"/>
+    <tableColumn id="5" name="部门补充：具体流程/文件/风险点"/>
+    <tableColumn id="6" name="培训触发（初稿）"/>
+    <tableColumn id="7" name="建议确认方式（初稿）"/>
+    <tableColumn id="8" name="能力/培训结果定义（待确认）"/>
+    <tableColumn id="9" name="责任角色（待确认）"/>
+    <tableColumn id="10" name="复核/频次（待确认）"/>
+    <tableColumn id="11" name="状态"/>
+    <tableColumn id="12" name="部门修订意见/证据位置"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_岗位能力矩阵" displayName="T_岗位能力矩阵" ref="A1:K2" headerRowCount="1">
   <autoFilter ref="A1:K2"/>
   <tableColumns count="11">
     <tableColumn id="1" name="岗位ID"/>
@@ -468,6 +538,700 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="66" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>模块编号</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>培训模块</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>适用对象（初稿）</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>通用目标/内容（部门需修订）</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>部门补充：具体流程/文件/风险点</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>培训触发（初稿）</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>建议确认方式（初稿）</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>能力/培训结果定义（待确认）</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>责任角色（待确认）</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>复核/频次（待确认）</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>部门修订意见/证据位置</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>TR-01</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>公司入职与基本要求</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>所有新员工；转岗人员按需</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>了解公司基本情况、岗位归属、现场区域、沟通与异常报告渠道；具体内容由行政部补充。</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr"/>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>新入职、转岗或公司要求更新</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>讲解+问答/确认理解</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>完成必要介绍；未理解事项补充说明；具体完成标准待确认</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>行政部/用人部门（待确认）</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>新入职/转岗及内容变更触发；具体时限待确认</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr"/>
+    </row>
+    <row r="3" ht="72" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>TR-02</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>现场安全与应急基本认知</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>所有进入生产/仓储区域人员；外来人员按规则</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>识别本区域主要危险、个人防护要求、紧急停止/报警/疏散与报告路径；依据公司现场实际和适用要求补充，禁止用本模板代替设备安全培训。</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr"/>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>入职、进入新区域、风险/设施变化、事件复盘</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>现场讲解+理解确认；必要时演练（方式待确认）</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>关键安全事项理解并按公司指定方式确认；具体要求和限制待管理层确认</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>行政部协调；安全/部门责任人提供内容（待确认）</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>按风险和适用要求确定；周期/触发待确认</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4" ht="72" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>TR-03</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>产品、客户与图纸/版本识别</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>生产、工程、品质、仓储、采购等接触产品/材料岗位</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>认识扁平马达、无刷马达冲压外壳的产品类别；按受控资料识别上机壳/下机壳、产品编码、客户、图号及有效版本；具体料号和识别图由部门提供。</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>上岗、产品/图纸/客户要求变更</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>资料讲解+样件/图纸识别考核（样件与标准须经批准）</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>能够按受控资料识别当前任务所需产品/版本；样件与判定标准待部门确认</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>工程技术组/品质部/生产部（待确认）</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>新产品、版本或要求变化触发；复核频次待确认</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr"/>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>TR-04</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>生产任务、材料与批次追溯</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>生产、仓储、采购、品质相关岗位</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>理解工单/生产任务、材料牌号规格、材料批次、标签、领料/余料记录之间的关联；以公司批准资料为准，不使用本模板设定材料参数。</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>新岗、材料/产品/流程变化、异常后补训</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>记录走查/现场实物识别（按部门批准方式）</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>能够正确识别任务、材料及批次记录；“三项一致”等公司定义待确认</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>生产部/仓储组/采购组/品质部（待确认）</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>变更或异常��发；频次待确认</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>TR-05</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>连续模基本结构、换模/试模与模具异常</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>工程技术、模具维修、生产相关岗位；按职责区分</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>认识本公司连续模及工位/零件标识、换模交接、试模记录、异常上报和维修边界；具体模具结构、锁定/防护、安全步骤必须由公司设备与安全责任人按实际机台文件编制并批准。</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>岗位安排、模具/设备/方法变化、异常复盘</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>经授权人员讲解+受控现场示范/能力确认；不得自行练习危险操作</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>达到何种能力可独立/需监督、授权人及安全前提均待确认；本行不构成操作许可</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>模具维修组/工程技术组/生产部及安全责任人（待确认）</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>设备/模具或工艺变更、事件后复核；周期待确认</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>TR-06</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>冲压设备岗位安全与操作资格</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>仅适用于实际操作/调机岗位</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>必须使用对应机台的制造商资料、风险评估、公司批准作业文件和适用法规要求；培训内容、资格条件、停机/防护步骤均由合格责任人现场确认，本通用模板不提供机器操作指令或数值。</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>人员上岗、转岗、设备/防护/程序变化、事件后</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>由公司指定的合格人员依批准资料培训并实操评定</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>未完成公司规���的安全培训/授权前不得独立操作；授权条件和记录由管理层确认</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>生产部/设备或安全责任人（待确认）</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>法定/风险要求及公司规定待确认</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>TR-07</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>首件、过程检验与质量异常控制</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>生产、品质、工程、模具维修等相关岗位</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>依据有效图纸/检验标准理解首件、过程检查、异常报告、风险控制、隔离和复核接口；检查项目/频次/放行权限必须采用公司批准标准。</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>上岗、质量要求变化、异常/客户问题后</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>标准讲解+受控记录走查/必要实操</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>能按岗位职责记录或检验；隔离、放行和恢复权限待公司确认</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>品质部/生产部/工程技术组（待确认）</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>标准变更、异常后及部门确定的复核节点</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>TR-08</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>仓储收发存、状态与批次标识</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>仓储及相关收发/领料/品质岗位</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>识别材料/成品批次、状态、库位、待判/隔离标识、收发/退料记录及异常升级；状态定义和可用/放行权限待公司确认。</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>新岗、库位/标识/系统变化、异常后</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>现有真实记录走查+按批准规则现场确认</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>能按职责识别并记录批次/状态；状态转换权限待确认</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>仓储组/采购组/品质部（待确认）</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>变更及盘点/异常节点；频次待确认</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>TR-09</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>采购、供应商与客户要求传递</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>业务、采购、品质、生产、仓储等相关岗位</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>按职责识别客户订单、材料要求、图纸版本、交期、包装/标签及变更，并使用公司确定的有效信息传递路径；不得自行承诺变更。</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>新岗、客户/供应商要求或订单变更</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>真实订单记录走查/部门讲解</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>接收、评审、批准、生效和客户反馈责任待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>运营部/品质部/生产部/采购组（待确认）</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>订单/要求变化触发；频次待确认</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>TR-10</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>测量工具、检验方法与记录真实性</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>需使用量具或填写检验记录的岗位</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>按品质批准的量具清单、作业说明和图纸判定；识别量具状态、记录真实测量值及异常报告。具体量具、方法、判定标准由品质部填写。</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>岗位安排、检具/标准变化、测量异常</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>由品质指定人员示范+实际能力确认</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>量具选择、判定边界及合格标准待品质批准</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>品质部/相关部门（待确认）</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>检具/标准变更及风险触发；频次待确认</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>TR-11</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>办公室/职能岗位与记录保密</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>行政、运营、财务及接触客户/员工资料岗位</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>按岗位流程处理文件版本、客户/员工信息、记录保管、授权访问和异常升级；由各部门提供受控流程。</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>入职、岗位/系统/权限变化</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>流程讲解+记录/情境确认</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>访问权限与记录留存规则待公司确认</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>各职能部门/行政部（待确认）</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>权限或流程变更触发</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>待部门确认</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L12"/>
+  <dataValidations count="1">
+    <dataValidation sqref="K2:K12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"待部门确认,修订中,已确认,暂不适用"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.25" right="0.25" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K2"/>
@@ -602,6 +1366,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
+  <dataValidations count="2">
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"未评估,了解,需指导,需监督,可独立,不适用"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"待确认,可独立,需监督,未授权,暂停"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -609,7 +1381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3702,6 +4474,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M1"/>
+  <dataValidations count="3">
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"讲解,示范,实操,记录走查,线上学习,其他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"未考核,通过,未通过,待补训"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"未确认,可独立,需监督,暂不可上岗,不适用"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-27 00:14:53
</commit_message>
<xml_diff>
--- a/02_Areas/工作经历/鑫犇电子有限公司/04_行政部/人事/能力与培训模板.xlsx
+++ b/02_Areas/工作经历/鑫犇电子有限公司/04_行政部/人事/能力与培训模板.xlsx
@@ -12,8 +12,7 @@
     <sheet name="培训记录" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'培训模块与部门确认'!$A$1:$L$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'培训模块与部门确认'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'培训模块与部门确认'!$A$1:$N$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'岗位能力矩阵'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'培训记录'!$A$1:$M$1</definedName>
   </definedNames>
@@ -24,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +52,10 @@
     <font>
       <name val="Microsoft YaHei"/>
       <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -101,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -132,6 +135,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -211,21 +220,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_培训模块与部门确认" displayName="T_培训模块与部门确认" ref="A1:L12" headerRowCount="1">
-  <autoFilter ref="A1:L12"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_培训模块与部门确认" displayName="T_培训模块与部门确认" ref="A1:N12" headerRowCount="1">
+  <autoFilter ref="A1:N12"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="模块编号"/>
-    <tableColumn id="2" name="培训模块"/>
-    <tableColumn id="3" name="适用对象（初稿）"/>
-    <tableColumn id="4" name="通用目标/内容（部门需修订）"/>
-    <tableColumn id="5" name="部门补充：具体流程/文件/风险点"/>
-    <tableColumn id="6" name="培训触发（初稿）"/>
-    <tableColumn id="7" name="建议确认方式（初稿）"/>
-    <tableColumn id="8" name="能力/培训结果定义（待确认）"/>
-    <tableColumn id="9" name="责任角色（待确认）"/>
-    <tableColumn id="10" name="复核/频次（待确认）"/>
-    <tableColumn id="11" name="状态"/>
-    <tableColumn id="12" name="部门修订意见/证据位置"/>
+    <tableColumn id="2" name="模块名称（骨架）"/>
+    <tableColumn id="3" name="适用部门/岗位（由部门填写）"/>
+    <tableColumn id="4" name="培训目标（由部门填写）"/>
+    <tableColumn id="5" name="培训内容/任务（由部门填写）"/>
+    <tableColumn id="6" name="依据类型"/>
+    <tableColumn id="7" name="依据文件/版本/条款（由部门填写）"/>
+    <tableColumn id="8" name="风险与合规要求（由部门/管理层填写）"/>
+    <tableColumn id="9" name="培训/评价方式（由部门填写）"/>
+    <tableColumn id="10" name="责任角色/批准人（待确认）"/>
+    <tableColumn id="11" name="触发条件/复核周期（待确认）"/>
+    <tableColumn id="12" name="证据位置（由部门填写）"/>
+    <tableColumn id="13" name="状态"/>
+    <tableColumn id="14" name="部门修订意见"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -538,26 +549,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="66" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>模块编号</t>
@@ -565,663 +578,430 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>培训模块</t>
+          <t>模块名称（骨架）</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>适用对象（初稿）</t>
+          <t>适用部门/岗位（由部门填写）</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>通用目标/内容（部门需修订）</t>
+          <t>培训目标（由部门填写）</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>部门补充：具体流程/文件/风险点</t>
+          <t>培训内容/任务（由部门填写）</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>培训触发（初稿）</t>
+          <t>依据类型</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>建议确认方式（初稿）</t>
+          <t>依据文件/版本/条款（由部门填写）</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>能力/培训结果定义（待确认）</t>
+          <t>风险与合规要求（由部门/管理层填写）</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
-          <t>责任角色（待确认）</t>
+          <t>培训/评价方式（由部门填写）</t>
         </is>
       </c>
       <c r="J1" s="5" t="inlineStr">
         <is>
-          <t>复核/频次（待确认）</t>
+          <t>责任角色/批准人（待确认）</t>
         </is>
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
+          <t>触发条件/复核周期（待确认）</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>证据位置（由部门填写）</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
-        <is>
-          <t>部门修订意见/证据位置</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="72" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>部门修订意见</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>TR-01</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>公司入职与基本要求</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>所有新员工；转岗人员按需</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>了解公司基本情况、岗位归属、现场区域、沟通与异常报告渠道；具体内容由行政部补充。</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr"/>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>新入职、转岗或公司要求更新</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>讲解+问答/确认理解</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr">
-        <is>
-          <t>完成必要介绍；未理解事项补充说明；具体完成标准待确认</t>
-        </is>
-      </c>
-      <c r="I2" s="9" t="inlineStr">
-        <is>
-          <t>行政部/用人部门（待确认）</t>
-        </is>
-      </c>
-      <c r="J2" s="9" t="inlineStr">
-        <is>
-          <t>新入职/转岗及内容变更触发；具体时限待确认</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L2" s="8" t="inlineStr"/>
-    </row>
-    <row r="3" ht="72" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>入职与岗位基本要求</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr"/>
+      <c r="D2" s="13" t="inlineStr"/>
+      <c r="E2" s="13" t="inlineStr"/>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>内部管理/人事资料</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr"/>
+      <c r="H2" s="13" t="inlineStr"/>
+      <c r="I2" s="13" t="inlineStr"/>
+      <c r="J2" s="13" t="inlineStr"/>
+      <c r="K2" s="13" t="inlineStr"/>
+      <c r="L2" s="13" t="inlineStr"/>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N2" s="13" t="inlineStr"/>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>TR-02</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>现场安全与应急基本认知</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>所有进入生产/仓储区域人员；外来人员按规则</t>
-        </is>
-      </c>
-      <c r="D3" s="11" t="inlineStr">
-        <is>
-          <t>识别本区域主要危险、个人防护要求、紧急停止/报警/疏散与报告路径；依据公司现场实际和适用要求补充，禁止用本模板代替设备安全培训。</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr"/>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>入职、进入新区域、风险/设施变化、事件复盘</t>
-        </is>
-      </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>现场讲解+理解确认；必要时演练（方式待确认）</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>关键安全事项理解并按公司指定方式确认；具体要求和限制待管理层确认</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="inlineStr">
-        <is>
-          <t>行政部协调；安全/部门责任人提供内容（待确认）</t>
-        </is>
-      </c>
-      <c r="J3" s="9" t="inlineStr">
-        <is>
-          <t>按风险和适用要求确定；周期/触发待确认</t>
-        </is>
-      </c>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L3" s="8" t="inlineStr"/>
-    </row>
-    <row r="4" ht="72" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>现场安全、应急与劳动防护</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr"/>
+      <c r="D3" s="13" t="inlineStr"/>
+      <c r="E3" s="13" t="inlineStr"/>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>法规/政府规章、风险评估、公司安全文件</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr"/>
+      <c r="H3" s="13" t="inlineStr"/>
+      <c r="I3" s="13" t="inlineStr"/>
+      <c r="J3" s="13" t="inlineStr"/>
+      <c r="K3" s="13" t="inlineStr"/>
+      <c r="L3" s="13" t="inlineStr"/>
+      <c r="M3" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="inlineStr"/>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>TR-03</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>产品、客户与图纸/版本识别</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>生产、工程、品质、仓储、采购等接触产品/材料岗位</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>认识扁平马达、无刷马达冲压外壳的产品类别；按受控资料识别上机壳/下机壳、产品编码、客户、图号及有效版本；具体料号和识别图由部门提供。</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>上岗、产品/图纸/客户要求变更</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>资料讲解+样件/图纸识别考核（样件与标准须经批准）</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>能够按受控资料识别当前任务所需产品/版本；样件与判定标准待部门确认</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>工程技术组/品质部/生产部（待确认）</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>新产品、版本或要求变化触发；复核频次待确认</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L4" s="8" t="inlineStr"/>
-    </row>
-    <row r="5" ht="72" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>产品、客户、图纸与版本识别</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr"/>
+      <c r="D4" s="13" t="inlineStr"/>
+      <c r="E4" s="13" t="inlineStr"/>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>客户要求、受控图纸、公司产品资料</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr"/>
+      <c r="H4" s="13" t="inlineStr"/>
+      <c r="I4" s="13" t="inlineStr"/>
+      <c r="J4" s="13" t="inlineStr"/>
+      <c r="K4" s="13" t="inlineStr"/>
+      <c r="L4" s="13" t="inlineStr"/>
+      <c r="M4" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr"/>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>TR-04</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>生产任务、材料与批次追溯</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>生产、仓储、采购、品质相关岗位</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>理解工单/生产任务、材料牌号规格、材料批次、标签、领料/余料记录之间的关联；以公司批准资料为准，不使用本模板设定材料参数。</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>新岗、材料/产品/流程变化、异常后补训</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>记录走查/现场实物识别（按部门批准方式）</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>能够正确识别任务、材料及批次记录；“三项一致”等公司定义待确认</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
-        <is>
-          <t>生产部/仓储组/采购组/品质部（待确认）</t>
-        </is>
-      </c>
-      <c r="J5" s="9" t="inlineStr">
-        <is>
-          <t>变更或异常��发；频次待确认</t>
-        </is>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L5" s="8" t="inlineStr"/>
-    </row>
-    <row r="6" ht="72" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr"/>
+      <c r="D5" s="13" t="inlineStr"/>
+      <c r="E5" s="13" t="inlineStr"/>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>生产任务/领料/材料主数据/批次记录</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr"/>
+      <c r="H5" s="13" t="inlineStr"/>
+      <c r="I5" s="13" t="inlineStr"/>
+      <c r="J5" s="13" t="inlineStr"/>
+      <c r="K5" s="13" t="inlineStr"/>
+      <c r="L5" s="13" t="inlineStr"/>
+      <c r="M5" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr"/>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>TR-05</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>连续模基本结构、换模/试模与模具异常</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>工程技术、模具维修、生产相关岗位；按职责区分</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>认识本公司连续模及工位/零件标识、换模交接、试模记录、异常上报和维修边界；具体模具结构、锁定/防护、安全步骤必须由公司设备与安全责任人按实际机台文件编制并批准。</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>岗位安排、模具/设备/方法变化、异常复盘</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>经授权人员讲解+受控现场示范/能力确认；不得自行练习危险操作</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>达到何种能力可独立/需监督、授权人及安全前提均待确认；本行不构成操作许可</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>模具维修组/工程技术组/生产部及安全责任人（待确认）</t>
-        </is>
-      </c>
-      <c r="J6" s="9" t="inlineStr">
-        <is>
-          <t>设备/模具或工艺变更、事件后复核；周期待确认</t>
-        </is>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7" ht="72" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>连续模工位、换模、试模与模具异常</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr"/>
+      <c r="D6" s="13" t="inlineStr"/>
+      <c r="E6" s="13" t="inlineStr"/>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>模具/设备文件、风险评估、现场标准</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr"/>
+      <c r="H6" s="13" t="inlineStr"/>
+      <c r="I6" s="13" t="inlineStr"/>
+      <c r="J6" s="13" t="inlineStr"/>
+      <c r="K6" s="13" t="inlineStr"/>
+      <c r="L6" s="13" t="inlineStr"/>
+      <c r="M6" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>TR-06</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>冲压设备岗位安全与操作资格</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>仅适用于实际操作/调机岗位</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>必须使用对应机台的制造商资料、风险评估、公司批准作业文件和适用法规要求；培训内容、资格条件、停机/防护步骤均由合格责任人现场确认，本通用模板不提供机器操作指令或数值。</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>人员上岗、转岗、设备/防护/程序变化、事件后</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>由公司指定的合格人员依批准资料培训并实操评定</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>未完成公司规���的安全培训/授权前不得独立操作；授权条件和记录由管理层确认</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
-        <is>
-          <t>生产部/设备或安全责任人（待确认）</t>
-        </is>
-      </c>
-      <c r="J7" s="9" t="inlineStr">
-        <is>
-          <t>法定/风险要求及公司规定待确认</t>
-        </is>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8" ht="72" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr"/>
+      <c r="D7" s="13" t="inlineStr"/>
+      <c r="E7" s="13" t="inlineStr"/>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>设备说明书、风险评估、法规/资质要求</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr"/>
+      <c r="I7" s="13" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr"/>
+      <c r="K7" s="13" t="inlineStr"/>
+      <c r="L7" s="13" t="inlineStr"/>
+      <c r="M7" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>TR-07</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>首件、过程检验与质量异常控制</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>生产、品质、工程、模具维修等相关岗位</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>依据有效图纸/检验标准理解首件、过程检查、异常报告、风险控制、隔离和复核接口；检查项目/频次/放行权限必须采用公司批准标准。</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>上岗、质量要求变化、异常/客户问题后</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>标准讲解+受控记录走查/必要实操</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>能按岗位职责记录或检验；隔离、放行和恢复权限待公司确认</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>品质部/生产部/工程技术组（待确认）</t>
-        </is>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>标准变更、异常后及部门确定的复核节点</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L8" s="8" t="inlineStr"/>
-    </row>
-    <row r="9" ht="72" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>首件、过程检验与质量异常</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr"/>
+      <c r="D8" s="13" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr"/>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>图纸/检验标准、品质记录、异常处置规则</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr"/>
+      <c r="J8" s="13" t="inlineStr"/>
+      <c r="K8" s="13" t="inlineStr"/>
+      <c r="L8" s="13" t="inlineStr"/>
+      <c r="M8" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>TR-08</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>仓储收发存、状态与批次标识</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>仓储及相关收发/领料/品质岗位</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>识别材料/成品批次、状态、库位、待判/隔离标识、收发/退料记录及异常升级；状态定义和可用/放行权限待公司确认。</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>新岗、库位/标识/系统变化、异常后</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>现有真实记录走查+按批准规则现场确认</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>能按职责识别并记录批次/状态；状态转换权限待确认</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
-        <is>
-          <t>仓储组/采购组/品质部（待确认）</t>
-        </is>
-      </c>
-      <c r="J9" s="9" t="inlineStr">
-        <is>
-          <t>变更及盘点/异常节点；频次待确认</t>
-        </is>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L9" s="8" t="inlineStr"/>
-    </row>
-    <row r="10" ht="72" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>仓储收发、状态与批次标识</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr"/>
+      <c r="D9" s="13" t="inlineStr"/>
+      <c r="E9" s="13" t="inlineStr"/>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>仓储/采购/品质记录及状态定义</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr"/>
+      <c r="H9" s="13" t="inlineStr"/>
+      <c r="I9" s="13" t="inlineStr"/>
+      <c r="J9" s="13" t="inlineStr"/>
+      <c r="K9" s="13" t="inlineStr"/>
+      <c r="L9" s="13" t="inlineStr"/>
+      <c r="M9" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>TR-09</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>采购、供应商与客户要求传递</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>业务、采购、品质、生产、仓储等相关岗位</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>按职责识别客户订单、材料要求、图纸版本、交期、包装/标签及变更，并使用公司确定的有效信息传递路径；不得自行承诺变更。</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>新岗、客户/供应商要求或订单变更</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>真实订单记录走查/部门讲解</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
-        <is>
-          <t>接收、评审、批准、生效和客户反馈责任待确认</t>
-        </is>
-      </c>
-      <c r="I10" s="9" t="inlineStr">
-        <is>
-          <t>运营部/品质部/生产部/采购组（待确认）</t>
-        </is>
-      </c>
-      <c r="J10" s="9" t="inlineStr">
-        <is>
-          <t>订单/要求变化触发；频次待确认</t>
-        </is>
-      </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L10" s="8" t="inlineStr"/>
-    </row>
-    <row r="11" ht="72" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr"/>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>订单/客户要求/采购资料</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr"/>
+      <c r="J10" s="13" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr"/>
+      <c r="L10" s="13" t="inlineStr"/>
+      <c r="M10" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>TR-10</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>测量工具、检验方法与记录真实性</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>需使用量具或填写检验记录的岗位</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>按品质批准的量具清单、作业说明和图纸判定；识别量具状态、记录真实测量值及异常报告。具体量具、方法、判定标准由品质部填写。</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr"/>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>岗位安排、检具/标准变化、测量异常</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>由品质指定人员示范+实际能力确认</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>量具选择、判定边界及合格标准待品质批准</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>品质部/相关部门（待确认）</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
-        <is>
-          <t>检具/标准变更及风险触发；频次待确认</t>
-        </is>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L11" s="8" t="inlineStr"/>
-    </row>
-    <row r="12" ht="72" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>量具、检验方法与记录真实性</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr"/>
+      <c r="D11" s="13" t="inlineStr"/>
+      <c r="E11" s="13" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>图纸、检验标准、量具管理资料</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr"/>
+      <c r="H11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr"/>
+      <c r="J11" s="13" t="inlineStr"/>
+      <c r="K11" s="13" t="inlineStr"/>
+      <c r="L11" s="13" t="inlineStr"/>
+      <c r="M11" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="inlineStr"/>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>TR-11</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>办公室/职能岗位与记录保密</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>行政、运营、财务及接触客户/员工资料岗位</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>按岗位流程处理文件版本、客户/员工信息、记录保管、授权访问和异常升级；由各部门提供受控流程。</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>入职、岗位/系统/权限变化</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>流程讲解+记录/情境确认</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
-        <is>
-          <t>访问权限与记录留存规则待公司确认</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
-        <is>
-          <t>各职能部门/行政部（待确认）</t>
-        </is>
-      </c>
-      <c r="J12" s="9" t="inlineStr">
-        <is>
-          <t>权限或流程变更触发</t>
-        </is>
-      </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>待部门确认</t>
-        </is>
-      </c>
-      <c r="L12" s="8" t="inlineStr"/>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>职能岗位流程、信息与记录保护</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr"/>
+      <c r="D12" s="13" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>岗位流程、公司授权和适用法律要求</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr"/>
+      <c r="H12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr"/>
+      <c r="J12" s="13" t="inlineStr"/>
+      <c r="K12" s="13" t="inlineStr"/>
+      <c r="L12" s="13" t="inlineStr"/>
+      <c r="M12" s="12" t="inlineStr">
+        <is>
+          <t>待填写</t>
+        </is>
+      </c>
+      <c r="N12" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L12"/>
+  <autoFilter ref="A1:N12"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"待部门确认,修订中,已确认,暂不适用"</formula1>
+    <dataValidation sqref="M2:M12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"待填写,部门��订中,部门确认,管理层批准,不适用"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.25" right="0.25" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>